<commit_message>
added database xlsx, updated wrong class names, added CreateFoodCategoryDto, CreateFodItemDto, CreateFoodSuggestionDto, FoodSuggestionDto, same service interfaces. Implemented FoodItemService and FoodSuggestionService and added validators for CreateFoodCategory, CreatoFoodItem and CreateFoodSuggestion
</commit_message>
<xml_diff>
--- a/CalorieTracker.API/database.xlsx
+++ b/CalorieTracker.API/database.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7050ebdbfb3bd6a2/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7050ebdbfb3bd6a2/Desktop/CalorieTrackerApp/CalorieTracker.API/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="275" documentId="13_ncr:1_{1580DF95-631B-4749-B995-50146DE298ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9C0798B5-65EE-43F9-A502-801305C80242}"/>
+  <xr:revisionPtr revIDLastSave="293" documentId="13_ncr:1_{1580DF95-631B-4749-B995-50146DE298ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8AA2CFD3-39E2-4FF1-8298-14EE8950890F}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="850" uniqueCount="321">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="851" uniqueCount="323">
   <si>
     <t>Name</t>
   </si>
@@ -598,9 +598,6 @@
     <t>Месо и месне прерађевине</t>
   </si>
   <si>
-    <t>Бурек са Месо и месне прерађевинем</t>
-  </si>
-  <si>
     <t>Ливањски сир</t>
   </si>
   <si>
@@ -983,6 +980,15 @@
   </si>
   <si>
     <t>Primadonna</t>
+  </si>
+  <si>
+    <t>Бурек са месом</t>
+  </si>
+  <si>
+    <t>https://onefit.rs/tablica-kalorija/gotova-jela/burek-sa-mesom/</t>
+  </si>
+  <si>
+    <t>https://onefit.rs/tablica-kalorija/gotova-jela/burek-sa-sirom/</t>
   </si>
 </sst>
 </file>
@@ -1035,6 +1041,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3063,7 +3073,7 @@
     </row>
     <row r="62" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B62">
         <v>457</v>
@@ -3084,7 +3094,7 @@
         <v>25</v>
       </c>
       <c r="H62" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="J62" t="b">
         <v>0</v>
@@ -3098,7 +3108,7 @@
     </row>
     <row r="63" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B63">
         <v>444</v>
@@ -3119,7 +3129,7 @@
         <v>25</v>
       </c>
       <c r="H63" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="J63" t="b">
         <v>0</v>
@@ -3133,7 +3143,7 @@
     </row>
     <row r="64" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B64">
         <v>419</v>
@@ -3154,7 +3164,7 @@
         <v>25</v>
       </c>
       <c r="H64" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="J64" t="b">
         <v>0</v>
@@ -3168,7 +3178,7 @@
     </row>
     <row r="65" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B65">
         <v>54</v>
@@ -3189,7 +3199,7 @@
         <v>25</v>
       </c>
       <c r="H65" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="J65" t="b">
         <v>0</v>
@@ -3203,7 +3213,7 @@
     </row>
     <row r="66" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B66">
         <v>73</v>
@@ -3224,7 +3234,7 @@
         <v>25</v>
       </c>
       <c r="H66" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="J66" t="b">
         <v>0</v>
@@ -3238,7 +3248,7 @@
     </row>
     <row r="67" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B67">
         <v>382</v>
@@ -3259,7 +3269,7 @@
         <v>101</v>
       </c>
       <c r="H67" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="J67" t="b">
         <v>0</v>
@@ -3273,7 +3283,7 @@
     </row>
     <row r="68" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B68">
         <v>114</v>
@@ -3294,7 +3304,7 @@
         <v>101</v>
       </c>
       <c r="H68" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="J68" t="b">
         <v>0</v>
@@ -3398,7 +3408,7 @@
     </row>
     <row r="72" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B72">
         <v>82</v>
@@ -3419,7 +3429,7 @@
         <v>25</v>
       </c>
       <c r="H72" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="J72" t="b">
         <v>0</v>
@@ -3433,7 +3443,7 @@
     </row>
     <row r="73" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B73">
         <v>78</v>
@@ -3454,7 +3464,7 @@
         <v>25</v>
       </c>
       <c r="H73" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="J73" t="b">
         <v>0</v>
@@ -3468,7 +3478,7 @@
     </row>
     <row r="74" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B74">
         <v>72</v>
@@ -3489,7 +3499,7 @@
         <v>25</v>
       </c>
       <c r="H74" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="J74" t="b">
         <v>0</v>
@@ -3503,7 +3513,7 @@
     </row>
     <row r="75" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B75">
         <v>70</v>
@@ -3524,7 +3534,7 @@
         <v>25</v>
       </c>
       <c r="H75" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="J75" t="b">
         <v>0</v>
@@ -3538,7 +3548,7 @@
     </row>
     <row r="76" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B76">
         <v>55</v>
@@ -3559,7 +3569,7 @@
         <v>25</v>
       </c>
       <c r="H76" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="J76" t="b">
         <v>0</v>
@@ -3573,7 +3583,7 @@
     </row>
     <row r="77" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B77">
         <v>58</v>
@@ -3594,7 +3604,7 @@
         <v>25</v>
       </c>
       <c r="H77" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="J77" t="b">
         <v>0</v>
@@ -3608,7 +3618,7 @@
     </row>
     <row r="78" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B78">
         <v>61</v>
@@ -3629,7 +3639,7 @@
         <v>25</v>
       </c>
       <c r="H78" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="J78" t="b">
         <v>0</v>
@@ -3643,7 +3653,7 @@
     </row>
     <row r="79" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B79">
         <v>58</v>
@@ -3664,7 +3674,7 @@
         <v>25</v>
       </c>
       <c r="H79" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="J79" t="b">
         <v>0</v>
@@ -3742,7 +3752,7 @@
     </row>
     <row r="82" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B82">
         <v>56</v>
@@ -3763,7 +3773,7 @@
         <v>25</v>
       </c>
       <c r="H82" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="J82" t="b">
         <v>0</v>
@@ -3809,7 +3819,7 @@
     </row>
     <row r="84" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B84">
         <v>228</v>
@@ -3830,7 +3840,7 @@
         <v>49</v>
       </c>
       <c r="H84" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="J84" t="b">
         <v>1</v>
@@ -3844,7 +3854,7 @@
     </row>
     <row r="85" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B85">
         <v>239</v>
@@ -3865,7 +3875,7 @@
         <v>49</v>
       </c>
       <c r="H85" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="J85" t="b">
         <v>1</v>
@@ -3879,7 +3889,7 @@
     </row>
     <row r="86" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B86">
         <v>91</v>
@@ -3900,7 +3910,7 @@
         <v>49</v>
       </c>
       <c r="H86" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="J86" t="b">
         <v>1</v>
@@ -3914,7 +3924,7 @@
     </row>
     <row r="87" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B87">
         <v>180</v>
@@ -3935,7 +3945,7 @@
         <v>49</v>
       </c>
       <c r="H87" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="J87" t="b">
         <v>1</v>
@@ -3949,7 +3959,7 @@
     </row>
     <row r="88" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B88">
         <v>345</v>
@@ -3970,7 +3980,7 @@
         <v>92</v>
       </c>
       <c r="H88" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="J88" t="b">
         <v>0</v>
@@ -3984,7 +3994,7 @@
     </row>
     <row r="89" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B89">
         <v>510</v>
@@ -4002,7 +4012,7 @@
         <v>25</v>
       </c>
       <c r="H89" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="J89" t="b">
         <v>0</v>
@@ -4013,7 +4023,7 @@
     </row>
     <row r="90" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B90">
         <v>77</v>
@@ -4034,7 +4044,7 @@
         <v>111</v>
       </c>
       <c r="H90" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="J90" t="b">
         <v>0</v>
@@ -4121,7 +4131,7 @@
         <v>108</v>
       </c>
       <c r="H93" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="J93" t="b">
         <v>0</v>
@@ -4156,7 +4166,7 @@
         <v>108</v>
       </c>
       <c r="H94" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="J94" t="b">
         <v>0</v>
@@ -4170,7 +4180,7 @@
     </row>
     <row r="95" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B95">
         <v>406.7</v>
@@ -4191,7 +4201,7 @@
         <v>101</v>
       </c>
       <c r="H95" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="J95" t="b">
         <v>0</v>
@@ -4205,7 +4215,7 @@
     </row>
     <row r="96" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B96">
         <v>406.7</v>
@@ -4226,7 +4236,7 @@
         <v>101</v>
       </c>
       <c r="H96" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="J96" t="b">
         <v>0</v>
@@ -4240,7 +4250,7 @@
     </row>
     <row r="97" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B97">
         <v>63</v>
@@ -4261,7 +4271,7 @@
         <v>111</v>
       </c>
       <c r="H97" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="J97" t="b">
         <v>0</v>
@@ -4275,7 +4285,7 @@
     </row>
     <row r="98" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B98">
         <v>225</v>
@@ -4296,7 +4306,7 @@
         <v>25</v>
       </c>
       <c r="H98" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="J98" t="b">
         <v>0</v>
@@ -4502,7 +4512,7 @@
     </row>
     <row r="105" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B105">
         <v>62</v>
@@ -4523,7 +4533,7 @@
         <v>25</v>
       </c>
       <c r="H105" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="J105" t="b">
         <v>0</v>
@@ -4537,7 +4547,7 @@
     </row>
     <row r="106" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B106">
         <v>60</v>
@@ -4558,7 +4568,7 @@
         <v>92</v>
       </c>
       <c r="H106" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="J106" t="b">
         <v>0</v>
@@ -4572,7 +4582,7 @@
     </row>
     <row r="107" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B107">
         <v>154</v>
@@ -4593,7 +4603,7 @@
         <v>111</v>
       </c>
       <c r="H107" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="J107" t="b">
         <v>0</v>
@@ -4761,7 +4771,7 @@
     </row>
     <row r="113" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B113">
         <v>340</v>
@@ -4782,7 +4792,7 @@
         <v>114</v>
       </c>
       <c r="H113" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="J113" t="b">
         <v>0</v>
@@ -4796,22 +4806,22 @@
     </row>
     <row r="114" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>192</v>
+        <v>320</v>
       </c>
       <c r="B114">
-        <v>340</v>
+        <v>260</v>
       </c>
       <c r="C114">
-        <v>11</v>
+        <v>7.2</v>
       </c>
       <c r="D114">
-        <v>30</v>
+        <v>27.2</v>
       </c>
       <c r="E114">
-        <v>20</v>
+        <v>17.3</v>
       </c>
       <c r="F114" t="s">
-        <v>135</v>
+        <v>321</v>
       </c>
       <c r="G114" t="s">
         <v>114</v>
@@ -4863,19 +4873,19 @@
         <v>137</v>
       </c>
       <c r="B116">
-        <v>310</v>
+        <v>246</v>
       </c>
       <c r="C116">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D116">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="E116">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="F116" t="s">
-        <v>135</v>
+        <v>322</v>
       </c>
       <c r="G116" t="s">
         <v>114</v>
@@ -4927,22 +4937,25 @@
         <v>139</v>
       </c>
       <c r="B118">
-        <v>350</v>
+        <v>229</v>
       </c>
       <c r="C118">
-        <v>7</v>
+        <v>7.1</v>
       </c>
       <c r="D118">
-        <v>35</v>
+        <v>52.6</v>
       </c>
       <c r="E118">
-        <v>18</v>
+        <v>6</v>
+      </c>
+      <c r="F118" t="s">
+        <v>135</v>
       </c>
       <c r="G118" t="s">
         <v>114</v>
       </c>
       <c r="J118" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K118" t="b">
         <v>1</v>
@@ -5174,7 +5187,7 @@
     </row>
     <row r="126" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B126">
         <v>250</v>
@@ -5195,7 +5208,7 @@
         <v>111</v>
       </c>
       <c r="H126" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="J126" t="b">
         <v>0</v>
@@ -5241,7 +5254,7 @@
     </row>
     <row r="128" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B128">
         <v>326</v>
@@ -5262,7 +5275,7 @@
         <v>114</v>
       </c>
       <c r="H128" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="J128" t="b">
         <v>0</v>
@@ -5308,7 +5321,7 @@
     </row>
     <row r="130" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B130">
         <v>136</v>
@@ -5329,7 +5342,7 @@
         <v>70</v>
       </c>
       <c r="H130" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="J130" t="b">
         <v>1</v>
@@ -5407,7 +5420,7 @@
     </row>
     <row r="133" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B133">
         <v>30</v>
@@ -5428,7 +5441,7 @@
         <v>70</v>
       </c>
       <c r="H133" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="J133" t="b">
         <v>1</v>
@@ -5538,7 +5551,7 @@
     </row>
     <row r="137" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B137">
         <v>358</v>
@@ -5559,7 +5572,7 @@
         <v>92</v>
       </c>
       <c r="H137" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="J137" t="b">
         <v>0</v>
@@ -5599,7 +5612,7 @@
     </row>
     <row r="139" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B139">
         <v>277</v>
@@ -5620,7 +5633,7 @@
         <v>161</v>
       </c>
       <c r="H139" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="J139" t="b">
         <v>0</v>
@@ -5698,7 +5711,7 @@
     </row>
     <row r="142" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B142">
         <v>373</v>
@@ -5719,7 +5732,7 @@
         <v>108</v>
       </c>
       <c r="H142" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="J142" t="b">
         <v>0</v>
@@ -5733,7 +5746,7 @@
     </row>
     <row r="143" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B143">
         <v>370</v>
@@ -5754,7 +5767,7 @@
         <v>108</v>
       </c>
       <c r="H143" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="J143" t="b">
         <v>0</v>
@@ -5768,7 +5781,7 @@
     </row>
     <row r="144" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B144">
         <v>158</v>
@@ -5789,7 +5802,7 @@
         <v>70</v>
       </c>
       <c r="H144" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="J144" t="b">
         <v>1</v>
@@ -5803,7 +5816,7 @@
     </row>
     <row r="145" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B145">
         <v>48</v>
@@ -5824,7 +5837,7 @@
         <v>111</v>
       </c>
       <c r="H145" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="J145" t="b">
         <v>0</v>
@@ -5870,7 +5883,7 @@
     </row>
     <row r="147" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B147">
         <v>289</v>
@@ -5891,7 +5904,7 @@
         <v>161</v>
       </c>
       <c r="H147" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="J147" t="b">
         <v>0</v>
@@ -5905,7 +5918,7 @@
     </row>
     <row r="148" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B148">
         <v>13</v>
@@ -5926,7 +5939,7 @@
         <v>70</v>
       </c>
       <c r="H148" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="J148" t="b">
         <v>1</v>
@@ -5972,7 +5985,7 @@
     </row>
     <row r="150" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B150">
         <v>75</v>
@@ -5993,7 +6006,7 @@
         <v>70</v>
       </c>
       <c r="H150" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="J150" t="b">
         <v>1</v>
@@ -6007,7 +6020,7 @@
     </row>
     <row r="151" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="B151">
         <v>240</v>
@@ -6028,7 +6041,7 @@
         <v>161</v>
       </c>
       <c r="H151" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="J151" t="b">
         <v>0</v>
@@ -6042,7 +6055,7 @@
     </row>
     <row r="152" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B152">
         <v>244</v>
@@ -6063,7 +6076,7 @@
         <v>49</v>
       </c>
       <c r="H152" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="J152" t="b">
         <v>1</v>
@@ -6077,7 +6090,7 @@
     </row>
     <row r="153" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B153">
         <v>712</v>
@@ -6098,7 +6111,7 @@
         <v>134</v>
       </c>
       <c r="H153" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="J153" t="b">
         <v>0</v>
@@ -6112,7 +6125,7 @@
     </row>
     <row r="154" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="B154">
         <v>828</v>
@@ -6133,7 +6146,7 @@
         <v>166</v>
       </c>
       <c r="H154" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="J154" t="b">
         <v>0</v>
@@ -6289,7 +6302,7 @@
     </row>
     <row r="160" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B160">
         <v>164</v>
@@ -6310,7 +6323,7 @@
         <v>191</v>
       </c>
       <c r="H160" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="J160" t="b">
         <v>0</v>
@@ -6324,7 +6337,7 @@
     </row>
     <row r="161" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B161">
         <v>65</v>
@@ -6345,7 +6358,7 @@
         <v>25</v>
       </c>
       <c r="H161" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="J161" t="b">
         <v>0</v>
@@ -6359,7 +6372,7 @@
     </row>
     <row r="162" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B162">
         <v>41</v>
@@ -6380,7 +6393,7 @@
         <v>25</v>
       </c>
       <c r="H162" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="J162" t="b">
         <v>0</v>
@@ -6394,7 +6407,7 @@
     </row>
     <row r="163" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B163">
         <v>61</v>
@@ -6415,7 +6428,7 @@
         <v>25</v>
       </c>
       <c r="H163" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="J163" t="b">
         <v>0</v>
@@ -6429,7 +6442,7 @@
     </row>
     <row r="164" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B164">
         <v>521</v>
@@ -6450,7 +6463,7 @@
         <v>108</v>
       </c>
       <c r="H164" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="J164" t="b">
         <v>0</v>
@@ -6464,7 +6477,7 @@
     </row>
     <row r="165" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B165">
         <v>64</v>
@@ -6485,7 +6498,7 @@
         <v>25</v>
       </c>
       <c r="H165" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="J165" t="b">
         <v>0</v>
@@ -6499,7 +6512,7 @@
     </row>
     <row r="166" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B166">
         <v>372</v>
@@ -6520,7 +6533,7 @@
         <v>108</v>
       </c>
       <c r="H166" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="J166" t="b">
         <v>0</v>
@@ -6534,7 +6547,7 @@
     </row>
     <row r="167" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="B167">
         <v>372</v>
@@ -6555,7 +6568,7 @@
         <v>108</v>
       </c>
       <c r="H167" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="J167" t="b">
         <v>0</v>
@@ -6569,7 +6582,7 @@
     </row>
     <row r="168" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B168">
         <v>328</v>
@@ -6590,7 +6603,7 @@
         <v>108</v>
       </c>
       <c r="H168" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="J168" t="b">
         <v>0</v>
@@ -6604,7 +6617,7 @@
     </row>
     <row r="169" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B169">
         <v>367</v>
@@ -6625,7 +6638,7 @@
         <v>108</v>
       </c>
       <c r="H169" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="J169" t="b">
         <v>0</v>
@@ -6671,7 +6684,7 @@
     </row>
     <row r="171" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B171">
         <v>183</v>
@@ -6692,7 +6705,7 @@
         <v>25</v>
       </c>
       <c r="H171" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="J171" t="b">
         <v>0</v>
@@ -6770,7 +6783,7 @@
     </row>
     <row r="174" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B174">
         <v>386</v>
@@ -6791,7 +6804,7 @@
         <v>92</v>
       </c>
       <c r="H174" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="J174" t="b">
         <v>0</v>
@@ -6869,7 +6882,7 @@
     </row>
     <row r="177" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="B177">
         <v>76</v>
@@ -6890,7 +6903,7 @@
         <v>25</v>
       </c>
       <c r="H177" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="J177" t="b">
         <v>0</v>
@@ -6904,7 +6917,7 @@
     </row>
     <row r="178" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B178">
         <v>383</v>
@@ -6925,7 +6938,7 @@
         <v>92</v>
       </c>
       <c r="H178" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="J178" t="b">
         <v>0</v>
@@ -6939,7 +6952,7 @@
     </row>
     <row r="179" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B179">
         <v>368</v>
@@ -6960,7 +6973,7 @@
         <v>49</v>
       </c>
       <c r="H179" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="J179" t="b">
         <v>1</v>
@@ -7006,7 +7019,7 @@
     </row>
     <row r="181" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B181">
         <v>85</v>
@@ -7027,7 +7040,7 @@
         <v>25</v>
       </c>
       <c r="H181" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="J181" t="b">
         <v>0</v>
@@ -7041,7 +7054,7 @@
     </row>
     <row r="182" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="B182">
         <v>212</v>
@@ -7062,7 +7075,7 @@
         <v>191</v>
       </c>
       <c r="H182" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="J182" t="b">
         <v>0</v>
@@ -7076,7 +7089,7 @@
     </row>
     <row r="183" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B183">
         <v>54</v>
@@ -7097,7 +7110,7 @@
         <v>25</v>
       </c>
       <c r="H183" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="J183" t="b">
         <v>0</v>
@@ -7143,7 +7156,7 @@
     </row>
     <row r="185" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="B185">
         <v>204</v>
@@ -7164,7 +7177,7 @@
         <v>25</v>
       </c>
       <c r="H185" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="J185" t="b">
         <v>0</v>
@@ -7178,7 +7191,7 @@
     </row>
     <row r="186" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="B186">
         <v>299</v>
@@ -7199,7 +7212,7 @@
         <v>191</v>
       </c>
       <c r="H186" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="J186" t="b">
         <v>0</v>
@@ -7213,7 +7226,7 @@
     </row>
     <row r="187" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="B187">
         <v>111</v>
@@ -7234,7 +7247,7 @@
         <v>25</v>
       </c>
       <c r="H187" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="J187" t="b">
         <v>0</v>
@@ -7376,7 +7389,7 @@
     </row>
     <row r="192" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="B192">
         <v>254</v>
@@ -7397,7 +7410,7 @@
         <v>114</v>
       </c>
       <c r="H192" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="J192" t="b">
         <v>0</v>
@@ -7443,7 +7456,7 @@
     </row>
     <row r="194" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="B194">
         <v>231</v>
@@ -7464,7 +7477,7 @@
         <v>161</v>
       </c>
       <c r="H194" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="J194" t="b">
         <v>0</v>
@@ -7542,7 +7555,7 @@
     </row>
     <row r="197" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="B197">
         <v>56</v>
@@ -7563,7 +7576,7 @@
         <v>92</v>
       </c>
       <c r="H197" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="J197" t="b">
         <v>0</v>
@@ -7609,7 +7622,7 @@
     </row>
     <row r="199" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B199">
         <v>199</v>
@@ -7630,7 +7643,7 @@
         <v>191</v>
       </c>
       <c r="H199" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="J199" t="b">
         <v>0</v>
@@ -7644,7 +7657,7 @@
     </row>
     <row r="200" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A200" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="B200">
         <v>132</v>
@@ -7665,7 +7678,7 @@
         <v>191</v>
       </c>
       <c r="H200" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="J200" t="b">
         <v>0</v>
@@ -7679,7 +7692,7 @@
     </row>
     <row r="201" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A201" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="B201">
         <v>27</v>
@@ -7700,7 +7713,7 @@
         <v>96</v>
       </c>
       <c r="H201" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J201" t="b">
         <v>0</v>
@@ -7714,7 +7727,7 @@
     </row>
     <row r="202" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A202" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B202">
         <v>50</v>
@@ -7735,7 +7748,7 @@
         <v>25</v>
       </c>
       <c r="H202" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="J202" t="b">
         <v>0</v>
@@ -7749,7 +7762,7 @@
     </row>
     <row r="203" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="B203">
         <v>567</v>
@@ -7770,7 +7783,7 @@
         <v>108</v>
       </c>
       <c r="H203" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="J203" t="b">
         <v>0</v>
@@ -7784,7 +7797,7 @@
     </row>
     <row r="204" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A204" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="B204">
         <v>421</v>
@@ -7805,7 +7818,7 @@
         <v>108</v>
       </c>
       <c r="H204" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="J204" t="b">
         <v>0</v>
@@ -7819,7 +7832,7 @@
     </row>
     <row r="205" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A205" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="B205">
         <v>436</v>
@@ -7840,7 +7853,7 @@
         <v>108</v>
       </c>
       <c r="H205" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="J205" t="b">
         <v>0</v>
@@ -7854,7 +7867,7 @@
     </row>
     <row r="206" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A206" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="B206">
         <v>87</v>
@@ -7875,7 +7888,7 @@
         <v>25</v>
       </c>
       <c r="H206" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="J206" t="b">
         <v>0</v>
@@ -7889,7 +7902,7 @@
     </row>
     <row r="207" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="B207">
         <v>220</v>
@@ -7910,7 +7923,7 @@
         <v>25</v>
       </c>
       <c r="H207" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="J207" t="b">
         <v>0</v>
@@ -7924,7 +7937,7 @@
     </row>
     <row r="208" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="B208">
         <v>215</v>
@@ -7945,7 +7958,7 @@
         <v>191</v>
       </c>
       <c r="H208" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="J208" t="b">
         <v>0</v>
@@ -7980,7 +7993,7 @@
         <v>25</v>
       </c>
       <c r="H209" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="J209" t="b">
         <v>0</v>
@@ -7994,7 +8007,7 @@
     </row>
     <row r="210" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A210" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="B210">
         <v>72</v>
@@ -8015,7 +8028,7 @@
         <v>25</v>
       </c>
       <c r="H210" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="J210" t="b">
         <v>0</v>
@@ -8029,7 +8042,7 @@
     </row>
     <row r="211" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A211" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B211">
         <v>64</v>
@@ -8050,7 +8063,7 @@
         <v>25</v>
       </c>
       <c r="H211" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="J211" t="b">
         <v>0</v>
@@ -8064,7 +8077,7 @@
     </row>
     <row r="212" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A212" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="B212">
         <v>828</v>
@@ -8085,7 +8098,7 @@
         <v>166</v>
       </c>
       <c r="H212" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="J212" t="b">
         <v>0</v>

</xml_diff>